<commit_message>
Đồng bộ hai website theo app bản 173 (cột 7 Tiếng Việt 2)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/docs/lop2/KHDH ca khoi - Lop 2.xlsx
+++ b/assets/docs/lop2/KHDH ca khoi - Lop 2.xlsx
@@ -741,11 +741,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1a: HS chọn bài đọc về thiếu nhi trong kho sách điện tử GV mở sẵn và nói vì sao chọn bài đó.</t>
-        </is>
-      </c>
+      <c r="H10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1013,12 +1009,7 @@
           <t>20</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1a: HS biết tìm kiếm nội dung đơn giản trong môi trường số; biết tìm đọc bài thơ, câu chuyện về ngày Tết trên nguồn học liệu số do GV cung cấp, chọn nội dung phù hợp và không bấm vào liên kết lạ.
-Tích hợp AI 2.A1.2: HS nhận biết công cụ AI như ChatGPT/Gemini có thể gợi ý lời chúc Tết hoặc sửa lỗi chính tả; HS chỉ dùng để tham khảo, tự viết bằng lời chân thành, không sao chép nguyên văn và không nhập thông tin riêng tư.</t>
-        </is>
-      </c>
+      <c r="H19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1228,11 +1219,7 @@
           <t>29</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1a: HS xác định được nhu cầu thông tin và thực hiện tìm kiếm đơn giản trong môi trường số dưới sự hướng dẫn; biết tìm bài thơ/câu chuyện thiếu nhi phù hợp, chọn nguồn đọc an toàn, rõ tên bài, tác giả hoặc địa chỉ nguồn.</t>
-        </is>
-      </c>
+      <c r="H26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1472,11 +1459,7 @@
           <t>39</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.2 CB1a: HS biết chọn nguồn thông tin số đơn giản, tin cậy và tôn trọng bản quyền khi tìm bài viết/hình ảnh về hoạt động thể thao; không tự ý tải hình ảnh lạ, không sao chép tùy tiện và biết ghi nhớ tên bài, nguồn đọc.</t>
-        </is>
-      </c>
+      <c r="H34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1719,11 +1702,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 2.2 CB1a: HS nêu được điểm giống nhau giữa tấm thiệp, lời cảm ơn viết trên giấy và tin nhắn gửi bằng điện thoại.</t>
-        </is>
-      </c>
+      <c r="H42" s="4" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -1992,12 +1971,7 @@
           <t>60</t>
         </is>
       </c>
-      <c r="H51" s="4" t="inlineStr">
-        <is>
-          <t>Tích hợp AI 2.A1.2: HS nhận biết AI có thể gợi ý từ ngữ/dàn ý khi viết về con vật, nhưng chỉ dùng để tham khảo; HS phải tự quan sát, tự viết bằng lời của mình, không nhập thông tin riêng tư của gia đình.
-Năng lực số 5.2 CB1b: HS nói ý theo từng ô của sơ đồ để GV gõ vào, rồi dựa vào dàn ý trên màn hình mà viết đoạn văn của mình.</t>
-        </is>
-      </c>
+      <c r="H51" s="4" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -2207,11 +2181,7 @@
           <t>69</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 3.1 CB1a: HS đọc bài viết được chiếu trên màn hình, nói được một câu kể rõ việc của bạn và một chỗ cần bổ sung.</t>
-        </is>
-      </c>
+      <c r="H58" s="4" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -2454,11 +2424,7 @@
           <t>79</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1b: HS quan sát ảnh phóng to và nêu được chi tiết mình sẽ đưa vào bài tả.</t>
-        </is>
-      </c>
+      <c r="H66" s="4" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -2882,12 +2848,7 @@
           <t>100</t>
         </is>
       </c>
-      <c r="H80" s="4" t="inlineStr">
-        <is>
-          <t>Tích hợp AI (2.A1.2): HS nhận biết AI có thể hỗ trợ gợi ý ý tưởng theo khung câu hỏi khi viết đoạn giới thiệu đồ dùng học tập; biết sử dụng gợi ý ở mức tham khảo, không chép máy móc.
-Năng lực số 5.2 CB1b: HS nói ý theo từng ô của sơ đồ để GV gõ vào, rồi dựa vào dàn ý trên màn hình mà viết đoạn văn của mình.</t>
-        </is>
-      </c>
+      <c r="H80" s="4" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -4895,11 +4856,7 @@
           <t>190</t>
         </is>
       </c>
-      <c r="H145" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1a: HS chọn bài đọc về thiếu nhi trong kho sách điện tử GV mở sẵn và nói vì sao chọn bài đó.</t>
-        </is>
-      </c>
+      <c r="H145" s="4" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -5146,11 +5103,7 @@
           <t>200</t>
         </is>
       </c>
-      <c r="H153" s="4" t="inlineStr">
-        <is>
-          <t>Tích hợp AI - YCCĐ 2.A2.1: HS biết mục đích của AI trong gia đình là hỗ trợ con người, giúp tiết kiệm thời gian, giảm một số công việc nhà; con người vẫn cần sử dụng đúng mục đích và kiểm tra kết quả.</t>
-        </is>
-      </c>
+      <c r="H153" s="4" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="inlineStr">
@@ -5873,11 +5826,7 @@
           <t>229-230</t>
         </is>
       </c>
-      <c r="H176" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 2.2 CB1a: HS nêu được điểm giống nhau giữa tấm thiệp, lời cảm ơn viết trên giấy và tin nhắn gửi bằng điện thoại.</t>
-        </is>
-      </c>
+      <c r="H176" s="4" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="inlineStr">
@@ -6316,11 +6265,7 @@
           <t>249-250</t>
         </is>
       </c>
-      <c r="H190" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 3.1 CB1a: HS đọc bài viết được chiếu trên màn hình, nói được một câu kể rõ việc của bạn và một chỗ cần bổ sung.</t>
-        </is>
-      </c>
+      <c r="H190" s="4" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="inlineStr">
@@ -6539,11 +6484,7 @@
           <t>259-260</t>
         </is>
       </c>
-      <c r="H197" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1b: HS quan sát ảnh phóng to và nêu được chi tiết mình sẽ đưa vào bài tả.</t>
-        </is>
-      </c>
+      <c r="H197" s="4" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="inlineStr">
@@ -7070,12 +7011,7 @@
           <t>289</t>
         </is>
       </c>
-      <c r="H214" s="4" t="inlineStr">
-        <is>
-          <t>Tích hợp năng lực số/an toàn thiết bị: Biết đọc một số thông tin đơn giản trên bản hướng dẫn sử dụng; nhận biết cần hỏi người lớn trước khi dùng thiết bị điện, thiết bị số.
-Tích hợp AI - YCCĐ 2.A3.2: Biết công cụ AI có thể gợi ý thông tin nhưng cần người lớn hướng dẫn, kiểm tra; không tự làm theo hướng dẫn nguy hiểm hoặc chia sẻ thông tin riêng tư.</t>
-        </is>
-      </c>
+      <c r="H214" s="4" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="inlineStr">
@@ -7315,11 +7251,7 @@
           <t>299</t>
         </is>
       </c>
-      <c r="H222" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 2.2 CB1a: HS nêu được vì sao phải kiểm tra tên người nhận trước khi gửi và vì sao mình cần nhờ bố mẹ gửi giúp.</t>
-        </is>
-      </c>
+      <c r="H222" s="4" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="inlineStr">
@@ -7805,11 +7737,7 @@
           <t>319</t>
         </is>
       </c>
-      <c r="H238" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 1.1 CB1b: HS quan sát ảnh phóng to và nêu được chi tiết mình sẽ đưa vào bài tả.</t>
-        </is>
-      </c>
+      <c r="H238" s="4" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
@@ -8049,11 +7977,7 @@
           <t>329</t>
         </is>
       </c>
-      <c r="H246" s="4" t="inlineStr">
-        <is>
-          <t>Năng lực số 5.2 CB1b: HS nói ý theo từng ô của sơ đồ để GV gõ vào, rồi dựa vào dàn ý trên màn hình mà viết đoạn văn của mình.</t>
-        </is>
-      </c>
+      <c r="H246" s="4" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="inlineStr">

</xml_diff>